<commit_message>
Documentacion de la Fase 2 y carta Gantt actualizada
Gestion/2.1_DiarioReflexion_Fase2_Bastian_Bustamante.docx
  Diario de reflexion individual.

Gestion/2.4_Fase2_DesarrolloProyecto_FiadoNFC.docx
  Guia grupal de avance: resumen, plan de trabajo con catorce actividades y su
  estado real, factores que facilitaron y dificultaron, ajustes al plan y
  actividades no iniciadas con su estrategia.

Gestion/Carta_Gantt_FiadoNFC.xlsx
  Fases 1 a 4 cerradas al 100%. La segunda demostracion quedo en su fecha real
  (28-09) y no en la estimada. Se agregan dos fases nacidas de la
  retroalimentacion docente: Fase 5 con limite de credito, boleta asociada al
  movimiento y modo oscuro; y Fase 6 con el panel de indicadores, el modo sin
  conexion y el cierre.

El panel de indicadores quedo planificado con holgura y no para esta entrega,
siguiendo la indicacion del docente de tenerlo presente para los proximos
sprints.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gestion/Carta_Gantt_FiadoNFC.xlsx
+++ b/Gestion/Carta_Gantt_FiadoNFC.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="19200" windowHeight="5670" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gestión Proyecto Carta Gantt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestión Proyecto Carta Gantt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" concurrentCalc="0"/>
@@ -15,10 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy;@"/>
     <numFmt numFmtId="166" formatCode="DD-MM-YYYY"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -255,12 +256,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F29900"/>
+        <fgColor rgb="002E5EAA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5EAA"/>
+        <fgColor rgb="00F29900"/>
       </patternFill>
     </fill>
   </fills>
@@ -1305,10 +1306,6 @@
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="23" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
@@ -1318,13 +1315,17 @@
     <xf numFmtId="166" fontId="5" fillId="13" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="23" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1530,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:CP46"/>
+  <dimension ref="B1:CP53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.84375" defaultRowHeight="15.5"/>
   <cols>
     <col width="2.4609375" customWidth="1" min="1" max="1"/>
@@ -1572,7 +1573,7 @@
       </c>
       <c r="C2" s="66" t="inlineStr">
         <is>
-          <t>Fiado NFC - Registro de fiado con llavero NFC para almacenes de barrio</t>
+          <t>Fiado NFC - Registro de fiado con llavero NFC para negocios de barrio</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1597,7 @@
       </c>
       <c r="C4" s="60" t="inlineStr">
         <is>
-          <t>Almacén de barrio (cliente piloto: Botillería Don Bastián)</t>
+          <t>Negocio de barrio (cliente piloto)</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1608,7 @@
         </is>
       </c>
       <c r="C5" s="113" t="n">
-        <v>46286</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="6" ht="18" customFormat="1" customHeight="1" s="1" thickBot="1">
@@ -2611,7 +2612,7 @@
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>Validación del caso de uso con almacén de barrio</t>
+          <t>Validación del caso de uso con un negocio de barrio</t>
         </is>
       </c>
       <c r="D12" s="45" t="inlineStr">
@@ -3637,7 +3638,7 @@
       </c>
       <c r="C21" s="42" t="inlineStr">
         <is>
-          <t>Políticas de seguridad por fila, revocación del rol público y función del portal</t>
+          <t>Políticas de seguridad por fila y función del portal del cliente</t>
         </is>
       </c>
       <c r="D21" s="43" t="inlineStr">
@@ -4088,7 +4089,7 @@
       </c>
       <c r="C25" s="42" t="inlineStr">
         <is>
-          <t>Inicio de sesión del almacenero y pantalla de saldos</t>
+          <t>Inicio de sesión del vendedor y pantalla de saldos</t>
         </is>
       </c>
       <c r="D25" s="43" t="inlineStr">
@@ -4352,7 +4353,7 @@
       <c r="T27" s="21" t="n"/>
       <c r="U27" s="21" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="V27" s="21" t="n"/>
@@ -4361,7 +4362,7 @@
       <c r="Y27" s="22" t="n"/>
       <c r="Z27" s="22" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="AA27" s="22" t="n"/>
@@ -4556,7 +4557,7 @@
       </c>
       <c r="C29" s="144" t="inlineStr">
         <is>
-          <t>HITO: Demostración funcional ante el profesor</t>
+          <t>HITO: Primera demostración funcional (nota 6,0)</t>
         </is>
       </c>
       <c r="D29" s="45" t="inlineStr">
@@ -4795,7 +4796,7 @@
         <v>5</v>
       </c>
       <c r="H31" s="56" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="I31" s="51" t="n"/>
       <c r="J31" s="21" t="n"/>
@@ -4832,11 +4833,11 @@
       <c r="AO31" s="21" t="n"/>
       <c r="AP31" s="21" t="n"/>
       <c r="AQ31" s="21" t="n"/>
-      <c r="AR31" s="146" t="n"/>
-      <c r="AS31" s="146" t="n"/>
-      <c r="AT31" s="146" t="n"/>
-      <c r="AU31" s="146" t="n"/>
-      <c r="AV31" s="146" t="n"/>
+      <c r="AR31" s="135" t="n"/>
+      <c r="AS31" s="135" t="n"/>
+      <c r="AT31" s="135" t="n"/>
+      <c r="AU31" s="135" t="n"/>
+      <c r="AV31" s="135" t="n"/>
       <c r="AW31" s="20" t="n"/>
       <c r="AX31" s="21" t="n"/>
       <c r="AY31" s="21" t="n"/>
@@ -4897,20 +4898,20 @@
       </c>
       <c r="D32" s="43" t="inlineStr">
         <is>
-          <t>Marcelo y Felipe</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E32" s="132" t="n">
         <v>46287</v>
       </c>
       <c r="F32" s="133" t="n">
-        <v>46304</v>
+        <v>46293</v>
       </c>
       <c r="G32" s="75" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="H32" s="56" t="n">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="I32" s="51" t="n"/>
       <c r="J32" s="21" t="n"/>
@@ -4948,20 +4949,20 @@
       <c r="AP32" s="21" t="n"/>
       <c r="AQ32" s="21" t="n"/>
       <c r="AR32" s="23" t="n"/>
-      <c r="AS32" s="146" t="n"/>
-      <c r="AT32" s="146" t="n"/>
-      <c r="AU32" s="146" t="n"/>
-      <c r="AV32" s="146" t="n"/>
-      <c r="AW32" s="147" t="n"/>
-      <c r="AX32" s="146" t="n"/>
-      <c r="AY32" s="146" t="n"/>
-      <c r="AZ32" s="146" t="n"/>
-      <c r="BA32" s="146" t="n"/>
-      <c r="BB32" s="146" t="n"/>
-      <c r="BC32" s="146" t="n"/>
-      <c r="BD32" s="146" t="n"/>
-      <c r="BE32" s="146" t="n"/>
-      <c r="BF32" s="146" t="n"/>
+      <c r="AS32" s="135" t="n"/>
+      <c r="AT32" s="135" t="n"/>
+      <c r="AU32" s="135" t="n"/>
+      <c r="AV32" s="135" t="n"/>
+      <c r="AW32" s="143" t="n"/>
+      <c r="AX32" s="21" t="n"/>
+      <c r="AY32" s="21" t="n"/>
+      <c r="AZ32" s="21" t="n"/>
+      <c r="BA32" s="21" t="n"/>
+      <c r="BB32" s="32" t="n"/>
+      <c r="BC32" s="32" t="n"/>
+      <c r="BD32" s="32" t="n"/>
+      <c r="BE32" s="32" t="n"/>
+      <c r="BF32" s="32" t="n"/>
       <c r="BG32" s="21" t="n"/>
       <c r="BH32" s="21" t="n"/>
       <c r="BI32" s="21" t="n"/>
@@ -5016,16 +5017,16 @@
         </is>
       </c>
       <c r="E33" s="132" t="n">
-        <v>46293</v>
+        <v>46288</v>
       </c>
       <c r="F33" s="133" t="n">
-        <v>46310</v>
+        <v>46289</v>
       </c>
       <c r="G33" s="75" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H33" s="56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" s="51" t="n"/>
       <c r="J33" s="21" t="n"/>
@@ -5064,23 +5065,23 @@
       <c r="AQ33" s="21" t="n"/>
       <c r="AR33" s="23" t="n"/>
       <c r="AS33" s="23" t="n"/>
-      <c r="AT33" s="23" t="n"/>
-      <c r="AU33" s="23" t="n"/>
+      <c r="AT33" s="135" t="n"/>
+      <c r="AU33" s="135" t="n"/>
       <c r="AV33" s="23" t="n"/>
-      <c r="AW33" s="148" t="n"/>
-      <c r="AX33" s="149" t="n"/>
-      <c r="AY33" s="149" t="n"/>
-      <c r="AZ33" s="149" t="n"/>
-      <c r="BA33" s="149" t="n"/>
-      <c r="BB33" s="149" t="n"/>
-      <c r="BC33" s="149" t="n"/>
-      <c r="BD33" s="149" t="n"/>
-      <c r="BE33" s="149" t="n"/>
-      <c r="BF33" s="149" t="n"/>
-      <c r="BG33" s="149" t="n"/>
-      <c r="BH33" s="149" t="n"/>
-      <c r="BI33" s="149" t="n"/>
-      <c r="BJ33" s="149" t="n"/>
+      <c r="AW33" s="20" t="n"/>
+      <c r="AX33" s="21" t="n"/>
+      <c r="AY33" s="21" t="n"/>
+      <c r="AZ33" s="21" t="n"/>
+      <c r="BA33" s="21" t="n"/>
+      <c r="BB33" s="32" t="n"/>
+      <c r="BC33" s="32" t="n"/>
+      <c r="BD33" s="32" t="n"/>
+      <c r="BE33" s="32" t="n"/>
+      <c r="BF33" s="32" t="n"/>
+      <c r="BG33" s="21" t="n"/>
+      <c r="BH33" s="21" t="n"/>
+      <c r="BI33" s="21" t="n"/>
+      <c r="BJ33" s="21" t="n"/>
       <c r="BK33" s="21" t="n"/>
       <c r="BL33" s="32" t="n"/>
       <c r="BM33" s="32" t="n"/>
@@ -5120,9 +5121,9 @@
           <t>4.4</t>
         </is>
       </c>
-      <c r="C34" s="150" t="inlineStr">
-        <is>
-          <t>HITO: Segunda demostración funcional</t>
+      <c r="C34" s="146" t="inlineStr">
+        <is>
+          <t>HITO: Segunda demostración funcional (nota 6,5)</t>
         </is>
       </c>
       <c r="D34" s="49" t="inlineStr">
@@ -5130,17 +5131,17 @@
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E34" s="151" t="n">
-        <v>46314</v>
-      </c>
-      <c r="F34" s="152" t="n">
-        <v>46314</v>
+      <c r="E34" s="147" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F34" s="148" t="n">
+        <v>46293</v>
       </c>
       <c r="G34" s="76" t="n">
         <v>1</v>
       </c>
       <c r="H34" s="58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" s="52" t="n"/>
       <c r="J34" s="26" t="n"/>
@@ -5182,7 +5183,7 @@
       <c r="AT34" s="28" t="n"/>
       <c r="AU34" s="28" t="n"/>
       <c r="AV34" s="28" t="n"/>
-      <c r="AW34" s="25" t="n"/>
+      <c r="AW34" s="149" t="n"/>
       <c r="AX34" s="26" t="n"/>
       <c r="AY34" s="26" t="n"/>
       <c r="AZ34" s="26" t="n"/>
@@ -5197,7 +5198,7 @@
       <c r="BI34" s="26" t="n"/>
       <c r="BJ34" s="26" t="n"/>
       <c r="BK34" s="26" t="n"/>
-      <c r="BL34" s="153" t="n"/>
+      <c r="BL34" s="33" t="n"/>
       <c r="BM34" s="33" t="n"/>
       <c r="BN34" s="33" t="n"/>
       <c r="BO34" s="33" t="n"/>
@@ -5237,7 +5238,7 @@
       </c>
       <c r="C35" s="137" t="inlineStr">
         <is>
-          <t>FASE 5 - CIERRE Y ENTREGA FINAL</t>
+          <t>FASE 5 - MEJORAS PEDIDAS EN LA RETROALIMENTACIÓN</t>
         </is>
       </c>
       <c r="D35" s="138" t="n"/>
@@ -5343,7 +5344,7 @@
       </c>
       <c r="C36" s="42" t="inlineStr">
         <is>
-          <t>Modo sin conexión y sincronización de movimientos</t>
+          <t>Límite de crédito visible y aviso al superarlo</t>
         </is>
       </c>
       <c r="D36" s="43" t="inlineStr">
@@ -5352,13 +5353,13 @@
         </is>
       </c>
       <c r="E36" s="132" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F36" s="133" t="n">
         <v>46315</v>
       </c>
-      <c r="F36" s="133" t="n">
-        <v>46332</v>
-      </c>
       <c r="G36" s="75" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H36" s="56" t="n">
         <v>0</v>
@@ -5418,21 +5419,21 @@
       <c r="BI36" s="21" t="n"/>
       <c r="BJ36" s="21" t="n"/>
       <c r="BK36" s="21" t="n"/>
-      <c r="BL36" s="32" t="n"/>
-      <c r="BM36" s="149" t="n"/>
-      <c r="BN36" s="149" t="n"/>
-      <c r="BO36" s="149" t="n"/>
-      <c r="BP36" s="149" t="n"/>
-      <c r="BQ36" s="148" t="n"/>
-      <c r="BR36" s="149" t="n"/>
-      <c r="BS36" s="149" t="n"/>
-      <c r="BT36" s="149" t="n"/>
-      <c r="BU36" s="149" t="n"/>
-      <c r="BV36" s="149" t="n"/>
-      <c r="BW36" s="149" t="n"/>
-      <c r="BX36" s="149" t="n"/>
-      <c r="BY36" s="149" t="n"/>
-      <c r="BZ36" s="149" t="n"/>
+      <c r="BL36" s="150" t="n"/>
+      <c r="BM36" s="150" t="n"/>
+      <c r="BN36" s="32" t="n"/>
+      <c r="BO36" s="32" t="n"/>
+      <c r="BP36" s="32" t="n"/>
+      <c r="BQ36" s="20" t="n"/>
+      <c r="BR36" s="21" t="n"/>
+      <c r="BS36" s="21" t="n"/>
+      <c r="BT36" s="21" t="n"/>
+      <c r="BU36" s="21" t="n"/>
+      <c r="BV36" s="24" t="n"/>
+      <c r="BW36" s="24" t="n"/>
+      <c r="BX36" s="24" t="n"/>
+      <c r="BY36" s="24" t="n"/>
+      <c r="BZ36" s="24" t="n"/>
       <c r="CA36" s="21" t="n"/>
       <c r="CB36" s="21" t="n"/>
       <c r="CC36" s="21" t="n"/>
@@ -5458,22 +5459,22 @@
       </c>
       <c r="C37" s="42" t="inlineStr">
         <is>
-          <t>Pruebas integrales y corrección de hallazgos</t>
+          <t>Número de boleta asociado a cada movimiento</t>
         </is>
       </c>
       <c r="D37" s="43" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="E37" s="132" t="n">
-        <v>46328</v>
+        <v>46314</v>
       </c>
       <c r="F37" s="133" t="n">
-        <v>46339</v>
+        <v>46315</v>
       </c>
       <c r="G37" s="75" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H37" s="56" t="n">
         <v>0</v>
@@ -5533,8 +5534,8 @@
       <c r="BI37" s="21" t="n"/>
       <c r="BJ37" s="21" t="n"/>
       <c r="BK37" s="21" t="n"/>
-      <c r="BL37" s="32" t="n"/>
-      <c r="BM37" s="32" t="n"/>
+      <c r="BL37" s="150" t="n"/>
+      <c r="BM37" s="150" t="n"/>
       <c r="BN37" s="32" t="n"/>
       <c r="BO37" s="32" t="n"/>
       <c r="BP37" s="32" t="n"/>
@@ -5543,16 +5544,16 @@
       <c r="BS37" s="21" t="n"/>
       <c r="BT37" s="21" t="n"/>
       <c r="BU37" s="21" t="n"/>
-      <c r="BV37" s="149" t="n"/>
-      <c r="BW37" s="149" t="n"/>
-      <c r="BX37" s="149" t="n"/>
-      <c r="BY37" s="149" t="n"/>
-      <c r="BZ37" s="149" t="n"/>
-      <c r="CA37" s="149" t="n"/>
-      <c r="CB37" s="149" t="n"/>
-      <c r="CC37" s="149" t="n"/>
-      <c r="CD37" s="149" t="n"/>
-      <c r="CE37" s="149" t="n"/>
+      <c r="BV37" s="24" t="n"/>
+      <c r="BW37" s="24" t="n"/>
+      <c r="BX37" s="24" t="n"/>
+      <c r="BY37" s="24" t="n"/>
+      <c r="BZ37" s="24" t="n"/>
+      <c r="CA37" s="21" t="n"/>
+      <c r="CB37" s="21" t="n"/>
+      <c r="CC37" s="21" t="n"/>
+      <c r="CD37" s="21" t="n"/>
+      <c r="CE37" s="21" t="n"/>
       <c r="CF37" s="24" t="n"/>
       <c r="CG37" s="24" t="n"/>
       <c r="CH37" s="24" t="n"/>
@@ -5573,22 +5574,22 @@
       </c>
       <c r="C38" s="42" t="inlineStr">
         <is>
-          <t>Informe final y manual de usuario</t>
+          <t>Modo oscuro de la aplicación</t>
         </is>
       </c>
       <c r="D38" s="43" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Marcelo</t>
         </is>
       </c>
       <c r="E38" s="132" t="n">
-        <v>46335</v>
+        <v>46314</v>
       </c>
       <c r="F38" s="133" t="n">
-        <v>46346</v>
+        <v>46315</v>
       </c>
       <c r="G38" s="75" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H38" s="56" t="n">
         <v>0</v>
@@ -5648,8 +5649,8 @@
       <c r="BI38" s="21" t="n"/>
       <c r="BJ38" s="21" t="n"/>
       <c r="BK38" s="21" t="n"/>
-      <c r="BL38" s="32" t="n"/>
-      <c r="BM38" s="32" t="n"/>
+      <c r="BL38" s="150" t="n"/>
+      <c r="BM38" s="150" t="n"/>
       <c r="BN38" s="32" t="n"/>
       <c r="BO38" s="32" t="n"/>
       <c r="BP38" s="32" t="n"/>
@@ -5663,16 +5664,16 @@
       <c r="BX38" s="24" t="n"/>
       <c r="BY38" s="24" t="n"/>
       <c r="BZ38" s="24" t="n"/>
-      <c r="CA38" s="149" t="n"/>
-      <c r="CB38" s="149" t="n"/>
-      <c r="CC38" s="149" t="n"/>
-      <c r="CD38" s="149" t="n"/>
-      <c r="CE38" s="149" t="n"/>
-      <c r="CF38" s="149" t="n"/>
-      <c r="CG38" s="149" t="n"/>
-      <c r="CH38" s="149" t="n"/>
-      <c r="CI38" s="149" t="n"/>
-      <c r="CJ38" s="149" t="n"/>
+      <c r="CA38" s="21" t="n"/>
+      <c r="CB38" s="21" t="n"/>
+      <c r="CC38" s="21" t="n"/>
+      <c r="CD38" s="21" t="n"/>
+      <c r="CE38" s="21" t="n"/>
+      <c r="CF38" s="24" t="n"/>
+      <c r="CG38" s="24" t="n"/>
+      <c r="CH38" s="24" t="n"/>
+      <c r="CI38" s="24" t="n"/>
+      <c r="CJ38" s="24" t="n"/>
       <c r="CK38" s="20" t="n"/>
       <c r="CL38" s="21" t="n"/>
       <c r="CM38" s="21" t="n"/>
@@ -5686,9 +5687,9 @@
           <t>5.4</t>
         </is>
       </c>
-      <c r="C39" s="150" t="inlineStr">
-        <is>
-          <t>HITO: Presentación final</t>
+      <c r="C39" s="146" t="inlineStr">
+        <is>
+          <t>HITO: Entrega de avance de Fase 2</t>
         </is>
       </c>
       <c r="D39" s="49" t="inlineStr">
@@ -5696,14 +5697,14 @@
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E39" s="151" t="n">
-        <v>46349</v>
-      </c>
-      <c r="F39" s="152" t="n">
-        <v>46353</v>
+      <c r="E39" s="147" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F39" s="148" t="n">
+        <v>46315</v>
       </c>
       <c r="G39" s="76" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H39" s="58" t="n">
         <v>0</v>
@@ -5764,7 +5765,7 @@
       <c r="BJ39" s="26" t="n"/>
       <c r="BK39" s="26" t="n"/>
       <c r="BL39" s="33" t="n"/>
-      <c r="BM39" s="33" t="n"/>
+      <c r="BM39" s="151" t="n"/>
       <c r="BN39" s="33" t="n"/>
       <c r="BO39" s="33" t="n"/>
       <c r="BP39" s="33" t="n"/>
@@ -5788,59 +5789,274 @@
       <c r="CH39" s="29" t="n"/>
       <c r="CI39" s="29" t="n"/>
       <c r="CJ39" s="29" t="n"/>
-      <c r="CK39" s="154" t="n"/>
-      <c r="CL39" s="153" t="n"/>
-      <c r="CM39" s="153" t="n"/>
-      <c r="CN39" s="153" t="n"/>
-      <c r="CO39" s="153" t="n"/>
+      <c r="CK39" s="25" t="n"/>
+      <c r="CL39" s="26" t="n"/>
+      <c r="CM39" s="26" t="n"/>
+      <c r="CN39" s="26" t="n"/>
+      <c r="CO39" s="26" t="n"/>
       <c r="CP39" s="25" t="n"/>
     </row>
+    <row r="40">
+      <c r="B40" s="152" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C40" s="152" t="inlineStr">
+        <is>
+          <t>FASE 6 - PANEL DE INDICADORES Y CIERRE</t>
+        </is>
+      </c>
+      <c r="D40" s="152" t="n"/>
+      <c r="E40" s="152" t="n"/>
+      <c r="F40" s="152" t="n"/>
+      <c r="G40" s="152" t="n"/>
+      <c r="H40" s="152" t="n"/>
+    </row>
     <row r="41">
-      <c r="B41" s="155" t="inlineStr">
-        <is>
-          <t>LEYENDA</t>
-        </is>
-      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Panel de indicadores del negocio (dashboard)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E41" s="153" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F41" s="153" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G41" t="n">
+        <v>17</v>
+      </c>
+      <c r="H41" s="154" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN41" s="155" t="n"/>
+      <c r="BO41" s="155" t="n"/>
+      <c r="BP41" s="155" t="n"/>
+      <c r="BQ41" s="155" t="n"/>
+      <c r="BR41" s="155" t="n"/>
+      <c r="BS41" s="155" t="n"/>
+      <c r="BT41" s="155" t="n"/>
+      <c r="BU41" s="155" t="n"/>
+      <c r="BV41" s="155" t="n"/>
+      <c r="BW41" s="155" t="n"/>
+      <c r="BX41" s="155" t="n"/>
+      <c r="BY41" s="155" t="n"/>
+      <c r="BZ41" s="155" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="156" t="n"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Completado</t>
-        </is>
-      </c>
+          <t>Modo sin conexión y sincronización de movimientos</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Bastián</t>
+        </is>
+      </c>
+      <c r="E42" s="153" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F42" s="153" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G42" t="n">
+        <v>17</v>
+      </c>
+      <c r="H42" s="154" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN42" s="155" t="n"/>
+      <c r="BO42" s="155" t="n"/>
+      <c r="BP42" s="155" t="n"/>
+      <c r="BQ42" s="155" t="n"/>
+      <c r="BR42" s="155" t="n"/>
+      <c r="BS42" s="155" t="n"/>
+      <c r="BT42" s="155" t="n"/>
+      <c r="BU42" s="155" t="n"/>
+      <c r="BV42" s="155" t="n"/>
+      <c r="BW42" s="155" t="n"/>
+      <c r="BX42" s="155" t="n"/>
+      <c r="BY42" s="155" t="n"/>
+      <c r="BZ42" s="155" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="157" t="n"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>En curso</t>
-        </is>
-      </c>
+          <t>Pruebas integrales y corrección de hallazgos</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E43" s="153" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F43" s="153" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G43" t="n">
+        <v>12</v>
+      </c>
+      <c r="H43" s="154" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA43" s="155" t="n"/>
+      <c r="CB43" s="155" t="n"/>
+      <c r="CC43" s="155" t="n"/>
+      <c r="CD43" s="155" t="n"/>
+      <c r="CE43" s="155" t="n"/>
+      <c r="CF43" s="155" t="n"/>
+      <c r="CG43" s="155" t="n"/>
+      <c r="CH43" s="155" t="n"/>
+      <c r="CI43" s="155" t="n"/>
+      <c r="CJ43" s="155" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="158" t="n"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
+          <t>Informe final y manual de usuario</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E44" s="153" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F44" s="153" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G44" t="n">
+        <v>12</v>
+      </c>
+      <c r="H44" s="154" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA44" s="155" t="n"/>
+      <c r="CB44" s="155" t="n"/>
+      <c r="CC44" s="155" t="n"/>
+      <c r="CD44" s="155" t="n"/>
+      <c r="CE44" s="155" t="n"/>
+      <c r="CF44" s="155" t="n"/>
+      <c r="CG44" s="155" t="n"/>
+      <c r="CH44" s="155" t="n"/>
+      <c r="CI44" s="155" t="n"/>
+      <c r="CJ44" s="155" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="159" t="n"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Hito / Fase</t>
-        </is>
-      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="C45" s="156" t="inlineStr">
+        <is>
+          <t>HITO: Presentación final</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E45" s="153" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F45" s="153" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G45" t="n">
+        <v>5</v>
+      </c>
+      <c r="H45" s="154" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK45" s="157" t="n"/>
+      <c r="CL45" s="157" t="n"/>
+      <c r="CM45" s="157" t="n"/>
+      <c r="CN45" s="157" t="n"/>
+      <c r="CO45" s="157" t="n"/>
     </row>
     <row r="46" ht="19" customHeight="1">
-      <c r="B46" t="inlineStr">
+      <c r="C46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="156" t="inlineStr">
+        <is>
+          <t>LEYENDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="158" t="n"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="159" t="n"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="155" t="n"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="157" t="n"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Hito / Fase</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Semana 1 = lunes 03-08-2026. Las columnas cubren solo días hábiles (lunes a viernes).</t>
         </is>
       </c>
-      <c r="C46" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">

</xml_diff>